<commit_message>
Add deal template placeholders and field configuration for Hermes Garant
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/excel/Шаблон_сделки_ГермесГарант_Заполненный.xlsx
+++ b/excel/Шаблон_сделки_ГермесГарант_Заполненный.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="107">
   <si>
     <t>СДЕЛКА</t>
   </si>
@@ -31,6 +31,12 @@
     <t>14.07.2026</t>
   </si>
   <si>
+    <t>Дата окончания договора</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>Тип договора</t>
   </si>
   <si>
@@ -161,9 +167,6 @@
   </si>
   <si>
     <t>Материал стен</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>Год постройки</t>
@@ -719,7 +722,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B96"/>
+  <dimension ref="A1:B97"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -749,10 +752,10 @@
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="A4" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" t="s">
         <v>6</v>
       </c>
     </row>
@@ -784,55 +787,55 @@
       <c r="A8" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="3">
-        <v>150450</v>
+      <c r="B8" s="3" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="3" t="s">
         <v>15</v>
       </c>
+      <c r="B9" s="3">
+        <v>150450</v>
+      </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B10">
-        <v>1200</v>
+      <c r="B10" s="3" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B11">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12">
         <v>400</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="13" ht="17.25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B13"/>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+      <c r="B13" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="3" t="s">
+    </row>
+    <row r="14" ht="17.25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
         <v>22</v>
       </c>
+      <c r="B14" s="1"/>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
@@ -870,19 +873,19 @@
       <c r="A19" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="3"/>
+      <c r="B19" s="3" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>32</v>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="B20" s="3"/>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>34</v>
@@ -901,15 +904,15 @@
         <v>37</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -957,116 +960,118 @@
         <v>50</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="31" ht="17.25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B31" s="1"/>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" s="2" t="s">
+      <c r="B31" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32" ht="17.25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B32" s="3" t="s">
-        <v>53</v>
-      </c>
+      <c r="B32" s="1"/>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B33" s="3" t="s">
         <v>54</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34" s="3" t="s">
         <v>56</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B35" s="3" t="s">
         <v>58</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B36" s="3" t="s">
         <v>60</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B37" s="3" t="s">
         <v>62</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B38" s="3" t="s">
         <v>64</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B39" s="3" t="s">
         <v>66</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B40" s="3" t="s">
         <v>68</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B41" s="3" t="s">
         <v>70</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B42" s="3" t="s">
         <v>72</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B43" s="3" t="s">
         <v>74</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B44" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B44" s="3"/>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
@@ -1074,23 +1079,21 @@
       </c>
       <c r="B45" s="3"/>
     </row>
-    <row r="46" ht="17.25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" s="1" t="s">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B46" s="1"/>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B47" s="3" t="s">
+      <c r="B46" s="3"/>
+    </row>
+    <row r="47" ht="17.25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" s="1" t="s">
         <v>79</v>
       </c>
+      <c r="B47" s="1"/>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B48" s="3" t="s">
         <v>80</v>
@@ -1098,7 +1101,7 @@
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B49" s="3" t="s">
         <v>81</v>
@@ -1106,7 +1109,7 @@
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>82</v>
@@ -1114,23 +1117,23 @@
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>61</v>
+        <v>83</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B52" s="3" t="s">
         <v>62</v>
-      </c>
-      <c r="B52" s="3" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B53" s="3" t="s">
         <v>84</v>
@@ -1138,61 +1141,61 @@
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B55" s="3" t="s">
         <v>68</v>
-      </c>
-      <c r="B55" s="3" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>24</v>
+        <v>86</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>86</v>
+        <v>26</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B58" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B58" s="3" t="s">
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" s="2" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="59" ht="17.25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A59" s="1" t="s">
+      <c r="B59" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B59" s="1"/>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A60" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B60" s="3" t="s">
+    </row>
+    <row r="60" ht="17.25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" s="1" t="s">
         <v>90</v>
       </c>
+      <c r="B60" s="1"/>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B61" s="3" t="s">
         <v>91</v>
@@ -1200,7 +1203,7 @@
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B62" s="3" t="s">
         <v>92</v>
@@ -1208,31 +1211,31 @@
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>61</v>
+        <v>83</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B65" s="3" t="s">
         <v>62</v>
-      </c>
-      <c r="B65" s="3" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B66" s="3" t="s">
         <v>84</v>
@@ -1240,137 +1243,137 @@
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B68" s="3" t="s">
         <v>68</v>
-      </c>
-      <c r="B68" s="3" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>24</v>
+        <v>86</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>86</v>
+        <v>26</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B71" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B71" s="3"/>
-    </row>
-    <row r="72" ht="17.25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A72" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="B72" s="1"/>
-    </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A73" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B73" s="3"/>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B72" s="3"/>
+    </row>
+    <row r="73" ht="17.25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B73" s="1"/>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B74" s="3"/>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B75" s="3"/>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B76" s="3"/>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B77" s="3"/>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B78" s="3"/>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B79" s="3"/>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B80" s="3"/>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B81" s="3"/>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B82" s="3"/>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B83" s="3"/>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="B84" s="3"/>
     </row>
-    <row r="85" ht="17.25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A85" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="B85" s="1"/>
-    </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A86" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B86" s="3" t="s">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A85" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B85" s="3"/>
+    </row>
+    <row r="86" ht="17.25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A86" s="1" t="s">
         <v>95</v>
       </c>
+      <c r="B86" s="1"/>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B87" s="3" t="s">
         <v>96</v>
@@ -1378,7 +1381,7 @@
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B88" s="3" t="s">
         <v>97</v>
@@ -1386,7 +1389,7 @@
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B89" s="3" t="s">
         <v>98</v>
@@ -1394,7 +1397,7 @@
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B90" s="3" t="s">
         <v>99</v>
@@ -1402,7 +1405,7 @@
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B91" s="3" t="s">
         <v>100</v>
@@ -1410,7 +1413,7 @@
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B92" s="3" t="s">
         <v>101</v>
@@ -1418,7 +1421,7 @@
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B93" s="3" t="s">
         <v>102</v>
@@ -1426,7 +1429,7 @@
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B94" s="3" t="s">
         <v>103</v>
@@ -1434,7 +1437,7 @@
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B95" s="3" t="s">
         <v>104</v>
@@ -1442,21 +1445,29 @@
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B96" s="3" t="s">
         <v>105</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A97" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B97" s="3" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="A59:B59"/>
-    <mergeCell ref="A72:B72"/>
-    <mergeCell ref="A85:B85"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="A60:B60"/>
+    <mergeCell ref="A73:B73"/>
+    <mergeCell ref="A86:B86"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" sqref="B41">

</xml_diff>